<commit_message>
fix(catering-es-2.2): comida al 82 % (SPEC D4) y Tesorería sin «pan común»; landing: equilibrio en torno a 108 eventos
Mismos defectos que el m9 y el m8 del paellero, por la misma vía (a.py → ciclo.sh → cifras → docx):
neto año 1 39.297 → 39.540 €, DSCR 2,84 → 2,85, equilibrio 55 → 54 invitados/evento y 109 → 108 eventos/año
(caja 106 → 105), holgura de caja 23,7/24,3 → 23,8/24,4 %. Sin cambios: ventas 447.850 €, inversión 130.365 €
y préstamo. Gates del catering en verde (motor 13/13, D15, idempotencia, censo, no latinos, restos, prohibidos).
Paellero: la nota del ejemplo de empresa explica que el margen objetivo cambia por canal (autotest 336/336).
sha256 Mac = VPS en los 22 ficheros.

Via: Claude Code

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KriAdpMP6uaswtiVvqtBvP
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/plan-catering-tematico-eventos/plan-financiero-catering-tematico-eventos.xlsx
+++ b/astro-site/public/dl/plan-catering-tematico-eventos/plan-financiero-catering-tematico-eventos.xlsx
@@ -823,7 +823,7 @@
       </c>
       <c r="B9" s="65">
         <f>IFERROR(IF($B$5="","",$B$5*(1+SUMPRODUCT('PyG 3 Años'!$E$10:$E$11,'PyG 3 Años'!$G$10:$G$11))),"")</f>
-        <v>58.328061247499996</v>
+        <v>58.33410550000001</v>
       </c>
       <c r="C9" t="str">
         <f>IFERROR("Precio por invitado sin IVA más el IVA medio ponderado de tus líneas de venta: "&amp;TEXT(SUMPRODUCT('PyG 3 Años'!$E$10:$E$11,'PyG 3 Años'!$G$10:$G$11)*100,"0")&amp;" %. En el servicio de catering todo va al 10 % (art. 91.Uno.2.2.º de la Ley 37/1992, alcohol incluido); el alcohol que sale por drop-off mueve la media. Aquí va redondeado. Compáralo con el rango del sector, que va con IVA.","")</f>
@@ -844,7 +844,7 @@
         </is>
       </c>
       <c r="B11" s="64" t="n">
-        <v>0.8519</v>
+        <v>0.82</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -860,7 +860,7 @@
       </c>
       <c r="B12" s="66">
         <f>IFERROR(IF(COUNT(B11)=0,"",1-B11),"")</f>
-        <v>0.1481</v>
+        <v>0.18000000000000005</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -2541,19 +2541,19 @@
       </c>
       <c r="B10" s="32">
         <f>IFERROR(IF(B9="","",B9*$E$10),"")</f>
-        <v>381523.415</v>
+        <v>367237.0</v>
       </c>
       <c r="C10" s="32">
         <f>IFERROR(IF(C9="","",C9*$E$10),"")</f>
-        <v>427306.2248</v>
+        <v>411305.44</v>
       </c>
       <c r="D10" s="32">
         <f>IFERROR(IF(D9="","",D9*$E$10),"")</f>
-        <v>461490.7227840001</v>
+        <v>444209.87520000007</v>
       </c>
       <c r="E10" s="68">
         <f>IFERROR(IF('0. Supuestos'!$B$11="","",'0. Supuestos'!$B$11),"")</f>
-        <v>0.8519</v>
+        <v>0.82</v>
       </c>
       <c r="F10" s="28" t="inlineStr">
         <is>
@@ -2574,19 +2574,19 @@
       </c>
       <c r="B11" s="32">
         <f>IFERROR(IF(B9="","",B9*$E$11),"")</f>
-        <v>66326.585</v>
+        <v>80613.00000000003</v>
       </c>
       <c r="C11" s="32">
         <f>IFERROR(IF(C9="","",C9*$E$11),"")</f>
-        <v>74285.77520000002</v>
+        <v>90286.56000000004</v>
       </c>
       <c r="D11" s="32">
         <f>IFERROR(IF(D9="","",D9*$E$11),"")</f>
-        <v>80228.63721600002</v>
+        <v>97509.48480000005</v>
       </c>
       <c r="E11" s="68">
         <f>IFERROR(IF('0. Supuestos'!$B$12="","",'0. Supuestos'!$B$12),"")</f>
-        <v>0.1481</v>
+        <v>0.18000000000000005</v>
       </c>
       <c r="F11" s="28" t="inlineStr">
         <is>
@@ -2621,19 +2621,19 @@
       </c>
       <c r="B13" s="32">
         <f>IFERROR(IF(B9="","",B9*'0. Supuestos'!$B$11*'0. Supuestos'!$B$13),"")</f>
-        <v>114457.02449999998</v>
+        <v>110171.09999999999</v>
       </c>
       <c r="C13" s="32">
         <f>IFERROR(IF(C9="","",C9*'0. Supuestos'!$B$11*'0. Supuestos'!$B$13),"")</f>
-        <v>128191.86744</v>
+        <v>123391.632</v>
       </c>
       <c r="D13" s="32">
         <f>IFERROR(IF(D9="","",D9*'0. Supuestos'!$B$11*'0. Supuestos'!$B$13),"")</f>
-        <v>138447.21683520003</v>
+        <v>133262.96256</v>
       </c>
       <c r="E13" s="68">
         <f>IFERROR(B13/$B$9,"")</f>
-        <v>0.25556999999999996</v>
+        <v>0.24599999999999997</v>
       </c>
       <c r="F13" s="28" t="str">
         <f>IFERROR("Al "&amp;TEXT('0. Supuestos'!$B$13,"0%")&amp;" de las ventas de COMIDA, no del total: la bebida tiene su propia línea","")</f>
@@ -2653,19 +2653,19 @@
       </c>
       <c r="B14" s="32">
         <f>IFERROR(IF(B9="","",B9*'0. Supuestos'!$B$12*'0. Supuestos'!$B$14),"")</f>
-        <v>18571.443800000005</v>
+        <v>22571.64000000001</v>
       </c>
       <c r="C14" s="32">
         <f>IFERROR(IF(C9="","",C9*'0. Supuestos'!$B$12*'0. Supuestos'!$B$14),"")</f>
-        <v>20800.017056000008</v>
+        <v>25280.236800000013</v>
       </c>
       <c r="D14" s="32">
         <f>IFERROR(IF(D9="","",D9*'0. Supuestos'!$B$12*'0. Supuestos'!$B$14),"")</f>
-        <v>22464.018420480006</v>
+        <v>27302.655744000018</v>
       </c>
       <c r="E14" s="68">
         <f>IFERROR(B14/$B$9,"")</f>
-        <v>0.04146800000000001</v>
+        <v>0.05040000000000002</v>
       </c>
       <c r="F14" s="28" t="str">
         <f>IFERROR("Al "&amp;TEXT('0. Supuestos'!$B$14,"0%")&amp;" de las ventas de BEBIDA","")</f>
@@ -2811,19 +2811,19 @@
       </c>
       <c r="B19" s="26">
         <f>IFERROR(IF(B9="","",SUM(B13:B18)),"")</f>
-        <v>173334.96829999998</v>
+        <v>173049.24</v>
       </c>
       <c r="C19" s="26">
         <f>IFERROR(IF(C9="","",SUM(C13:C18)),"")</f>
-        <v>194135.164496</v>
+        <v>193815.14880000002</v>
       </c>
       <c r="D19" s="26">
         <f>IFERROR(IF(D9="","",SUM(D13:D18)),"")</f>
-        <v>209665.97765568004</v>
+        <v>209320.36070400005</v>
       </c>
       <c r="E19" s="67">
         <f>IFERROR(B19/$B$9,"")</f>
-        <v>0.38703799999999994</v>
+        <v>0.38639999999999997</v>
       </c>
       <c r="F19" s="28" t="n"/>
       <c r="G19" s="28" t="n"/>
@@ -2837,19 +2837,19 @@
       </c>
       <c r="B20" s="26">
         <f>IFERROR(IF(B9="","",B9-B19),"")</f>
-        <v>274515.03170000005</v>
+        <v>274800.76</v>
       </c>
       <c r="C20" s="26">
         <f>IFERROR(IF(C9="","",C9-C19),"")</f>
-        <v>307456.8355040001</v>
+        <v>307776.85120000003</v>
       </c>
       <c r="D20" s="26">
         <f>IFERROR(IF(D9="","",D9-D19),"")</f>
-        <v>332053.38234432007</v>
+        <v>332398.99929600005</v>
       </c>
       <c r="E20" s="67">
         <f>IFERROR(B20/$B$9,"")</f>
-        <v>0.6129620000000001</v>
+        <v>0.6136</v>
       </c>
       <c r="F20" s="28" t="n"/>
       <c r="G20" s="28" t="n"/>
@@ -3417,15 +3417,15 @@
       </c>
       <c r="B39" s="32">
         <f>IFERROR(IF(B9="","",SUMPRODUCT(B13:B18,G13:G18)),"")</f>
-        <v>22624.8275617</v>
+        <v>22882.268760000003</v>
       </c>
       <c r="C39" s="32">
         <f>IFERROR(IF(C9="","",SUMPRODUCT(C13:C18,G13:G18)),"")</f>
-        <v>25339.806869104006</v>
+        <v>25628.14101120001</v>
       </c>
       <c r="D39" s="32">
         <f>IFERROR(IF(D9="","",SUMPRODUCT(D13:D18,G13:G18)),"")</f>
-        <v>27366.99141863233</v>
+        <v>27678.39229209601</v>
       </c>
       <c r="E39" s="28" t="n"/>
       <c r="F39" s="28" t="inlineStr">
@@ -3467,19 +3467,19 @@
       </c>
       <c r="B41" s="26">
         <f>IFERROR(IF(B9="","",B20-B38),"")</f>
-        <v>46231.49170000004</v>
+        <v>46517.22</v>
       </c>
       <c r="C41" s="26">
         <f>IFERROR(IF(C9="","",C20-C38),"")</f>
-        <v>73173.29550400007</v>
+        <v>73493.31120000003</v>
       </c>
       <c r="D41" s="26">
         <f>IFERROR(IF(D9="","",D20-D38),"")</f>
-        <v>93037.04553308594</v>
+        <v>93382.66248476593</v>
       </c>
       <c r="E41" s="67">
         <f>IFERROR(B41/$B$9,"")</f>
-        <v>0.10322985754158769</v>
+        <v>0.10386785754158759</v>
       </c>
       <c r="F41" s="28" t="n"/>
       <c r="G41" s="28" t="n"/>
@@ -3520,15 +3520,15 @@
       </c>
       <c r="B43" s="32">
         <f>IFERROR(IF(B9="","",MAX(0,B41-B42)),"")</f>
-        <v>46231.49170000004</v>
+        <v>46517.22</v>
       </c>
       <c r="C43" s="32">
         <f>IFERROR(IF(C9="","",MAX(0,C41-C42)),"")</f>
-        <v>73173.29550400007</v>
+        <v>73493.31120000003</v>
       </c>
       <c r="D43" s="32">
         <f>IFERROR(IF(D9="","",MAX(0,D41-D42)),"")</f>
-        <v>93037.04553308594</v>
+        <v>93382.66248476593</v>
       </c>
       <c r="E43" s="28" t="n"/>
       <c r="F43" s="28" t="n"/>
@@ -3593,15 +3593,15 @@
       </c>
       <c r="B46" s="32">
         <f>IFERROR(IF(B9="","",IF(B45="",0,B43*B45)),"")</f>
-        <v>6934.723755000006</v>
+        <v>6977.583</v>
       </c>
       <c r="C46" s="32">
         <f>IFERROR(IF(C9="","",IF(C45="",0,C43*C45)),"")</f>
-        <v>10975.99432560001</v>
+        <v>11023.996680000004</v>
       </c>
       <c r="D46" s="32">
         <f>IFERROR(IF(D9="","",IF(D45="",0,D43*D45)),"")</f>
-        <v>23259.261383271485</v>
+        <v>23345.66562119148</v>
       </c>
       <c r="E46" s="28" t="n"/>
       <c r="F46" s="28" t="n"/>
@@ -3639,19 +3639,19 @@
       </c>
       <c r="B48" s="26">
         <f>IFERROR(IF(B9="","",B41-B46),"")</f>
-        <v>39296.767945000036</v>
+        <v>39539.637</v>
       </c>
       <c r="C48" s="26">
         <f>IFERROR(IF(C9="","",C41-C46),"")</f>
-        <v>62197.301178400056</v>
+        <v>62469.31452000002</v>
       </c>
       <c r="D48" s="26">
         <f>IFERROR(IF(D9="","",D41-D46),"")</f>
-        <v>69777.78414981446</v>
+        <v>70036.99686357444</v>
       </c>
       <c r="E48" s="67">
         <f>IFERROR(B48/$B$9,"")</f>
-        <v>0.08774537891034953</v>
+        <v>0.08828767891034946</v>
       </c>
       <c r="F48" s="28" t="n"/>
       <c r="G48" s="28" t="n"/>
@@ -3713,15 +3713,15 @@
       </c>
       <c r="B51" s="68">
         <f>IFERROR(IF(B9="","",B20/B9),"")</f>
-        <v>0.6129620000000001</v>
+        <v>0.6136</v>
       </c>
       <c r="C51" s="68">
         <f>IFERROR(IF(C9="","",C20/C9),"")</f>
-        <v>0.6129620000000001</v>
+        <v>0.6136</v>
       </c>
       <c r="D51" s="68">
         <f>IFERROR(IF(D9="","",D20/D9),"")</f>
-        <v>0.612962</v>
+        <v>0.6136</v>
       </c>
       <c r="E51" s="75" t="n">
         <v>0.6</v>
@@ -3742,15 +3742,15 @@
       </c>
       <c r="B52" s="32">
         <f>IFERROR(IF(B9="","",B13+B14),"")</f>
-        <v>133028.46829999998</v>
+        <v>132742.74</v>
       </c>
       <c r="C52" s="32">
         <f>IFERROR(IF(C9="","",C13+C14),"")</f>
-        <v>148991.884496</v>
+        <v>148671.8688</v>
       </c>
       <c r="D52" s="32">
         <f>IFERROR(IF(D9="","",D13+D14),"")</f>
-        <v>160911.23525568005</v>
+        <v>160565.61830400003</v>
       </c>
       <c r="E52" s="28" t="n"/>
       <c r="F52" s="28" t="n"/>
@@ -3765,15 +3765,15 @@
       </c>
       <c r="B53" s="68">
         <f>IFERROR(IF(B9="","",B52/B9),"")</f>
-        <v>0.29703799999999997</v>
+        <v>0.2964</v>
       </c>
       <c r="C53" s="68">
         <f>IFERROR(IF(C9="","",C52/C9),"")</f>
-        <v>0.29703799999999997</v>
+        <v>0.29639999999999994</v>
       </c>
       <c r="D53" s="68">
         <f>IFERROR(IF(D9="","",D52/D9),"")</f>
-        <v>0.297038</v>
+        <v>0.2964</v>
       </c>
       <c r="E53" s="75" t="n">
         <v>0.33</v>
@@ -3852,15 +3852,15 @@
       </c>
       <c r="B56" s="68">
         <f>IFERROR(IF(B9="","",B48/B9),"")</f>
-        <v>0.08774537891034953</v>
+        <v>0.08828767891034946</v>
       </c>
       <c r="C56" s="68">
         <f>IFERROR(IF(C9="","",C48/C9),"")</f>
-        <v>0.12399978703488103</v>
+        <v>0.12454208703488097</v>
       </c>
       <c r="D56" s="68">
         <f>IFERROR(IF(D9="","",D48/D9),"")</f>
-        <v>0.12880799414260263</v>
+        <v>0.1292864941426026</v>
       </c>
       <c r="E56" s="75" t="n">
         <v>0.04</v>
@@ -4170,15 +4170,15 @@
       </c>
       <c r="B9" s="70">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",'PyG 3 Años'!$B$19/('PyG 3 Años'!$B$6*'PyG 3 Años'!$B$8)),"")</f>
-        <v>20.513014</v>
+        <v>20.4792</v>
       </c>
       <c r="C9" s="70">
         <f>IFERROR(IF('PyG 3 Años'!$C$9="","",'PyG 3 Años'!$C$19/('PyG 3 Años'!$C$6*'PyG 3 Años'!$C$8)),"")</f>
-        <v>20.513014</v>
+        <v>20.4792</v>
       </c>
       <c r="D9" s="70">
         <f>IFERROR(IF('PyG 3 Años'!$D$9="","",'PyG 3 Años'!$D$19/('PyG 3 Años'!$D$6*'PyG 3 Años'!$D$8)),"")</f>
-        <v>20.513014</v>
+        <v>20.4792</v>
       </c>
       <c r="E9" s="28" t="inlineStr">
         <is>
@@ -4195,15 +4195,15 @@
       </c>
       <c r="B10" s="70">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",B8-B9),"")</f>
-        <v>32.486986</v>
+        <v>32.5208</v>
       </c>
       <c r="C10" s="70">
         <f>IFERROR(IF('PyG 3 Años'!$C$9="","",C8-C9),"")</f>
-        <v>32.486986</v>
+        <v>32.5208</v>
       </c>
       <c r="D10" s="70">
         <f>IFERROR(IF('PyG 3 Años'!$D$9="","",D8-D9),"")</f>
-        <v>32.486986</v>
+        <v>32.5208</v>
       </c>
       <c r="E10" s="28" t="inlineStr">
         <is>
@@ -4282,15 +4282,15 @@
       </c>
       <c r="B14" s="40">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",IF(B10&lt;=0,"",B6/B10)),"")</f>
-        <v>7026.922719146676</v>
+        <v>7019.616368601019</v>
       </c>
       <c r="C14" s="40">
         <f>IFERROR(IF('PyG 3 Años'!$C$9="","",IF(C10&lt;=0,"",C6/C10)),"")</f>
-        <v>7211.61205905651</v>
+        <v>7204.113674940346</v>
       </c>
       <c r="D14" s="40">
         <f>IFERROR(IF('PyG 3 Años'!$D$9="","",IF(D10&lt;=0,"",D6/D10)),"")</f>
-        <v>7357.294912222208</v>
+        <v>7349.645052127688</v>
       </c>
       <c r="E14" s="28" t="n"/>
       <c r="F14" s="28" t="n"/>
@@ -4303,15 +4303,15 @@
       </c>
       <c r="B15" s="44">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",B14/B11),"")</f>
-        <v>54.05325168574366</v>
+        <v>53.99704898923861</v>
       </c>
       <c r="C15" s="44">
         <f>IFERROR(IF('PyG 3 Años'!$C$9="","",C14/C11),"")</f>
-        <v>55.4739389158193</v>
+        <v>55.41625903800266</v>
       </c>
       <c r="D15" s="44">
         <f>IFERROR(IF('PyG 3 Años'!$D$9="","",D14/D11),"")</f>
-        <v>56.59457624786314</v>
+        <v>56.53573117021299</v>
       </c>
       <c r="E15" s="28" t="n"/>
       <c r="F15" s="28" t="n"/>
@@ -4324,15 +4324,15 @@
       </c>
       <c r="B16" s="26">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",B14*B8),"")</f>
-        <v>372426.90411477385</v>
+        <v>372039.667535854</v>
       </c>
       <c r="C16" s="26">
         <f>IFERROR(IF('PyG 3 Años'!$C$9="","",C14*C8),"")</f>
-        <v>382215.439129995</v>
+        <v>381818.02477183833</v>
       </c>
       <c r="D16" s="26">
         <f>IFERROR(IF('PyG 3 Años'!$D$9="","",D14*D8),"")</f>
-        <v>389936.63034777704</v>
+        <v>389531.1877627675</v>
       </c>
       <c r="E16" s="28" t="n"/>
       <c r="F16" s="28" t="n"/>
@@ -4382,15 +4382,15 @@
       </c>
       <c r="B19" s="40">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",IF(B10&lt;=0,"",B18/B10)),"")</f>
-        <v>6831.690696083656</v>
+        <v>6824.587341024821</v>
       </c>
       <c r="C19" s="40">
         <f>IFERROR(IF('PyG 3 Años'!$C$9="","",IF(C10&lt;=0,"",C18/C10)),"")</f>
-        <v>7616.47983205709</v>
+        <v>7608.560480471607</v>
       </c>
       <c r="D19" s="40">
         <f>IFERROR(IF('PyG 3 Años'!$D$9="","",IF(D10&lt;=0,"",D18/D10)),"")</f>
-        <v>7801.169171966923</v>
+        <v>7793.057786810934</v>
       </c>
       <c r="E19" s="28" t="n"/>
       <c r="F19" s="28" t="n"/>
@@ -4403,15 +4403,15 @@
       </c>
       <c r="B20" s="45">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",B19/B11),"")</f>
-        <v>52.5514668929512</v>
+        <v>52.49682570019093</v>
       </c>
       <c r="C20" s="45">
         <f>IFERROR(IF('PyG 3 Años'!$C$9="","",C19/C11),"")</f>
-        <v>58.58830640043915</v>
+        <v>58.52738831132005</v>
       </c>
       <c r="D20" s="45">
         <f>IFERROR(IF('PyG 3 Años'!$D$9="","",D19/D11),"")</f>
-        <v>60.008993630514794</v>
+        <v>59.94659836008411</v>
       </c>
       <c r="E20" s="28" t="n"/>
       <c r="F20" s="28" t="n"/>
@@ -4424,15 +4424,15 @@
       </c>
       <c r="B21" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",B19*B8),"")</f>
-        <v>362079.6068924338</v>
+        <v>361703.12907431554</v>
       </c>
       <c r="C21" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$C$9="","",C19*C8),"")</f>
-        <v>403673.43109902577</v>
+        <v>403253.7054649952</v>
       </c>
       <c r="D21" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$D$9="","",D19*D8),"")</f>
-        <v>413461.9661142469</v>
+        <v>413032.0627009795</v>
       </c>
       <c r="E21" s="28" t="n"/>
       <c r="F21" s="28" t="n"/>
@@ -4478,15 +4478,15 @@
       </c>
       <c r="B24" s="68">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",B23/B20-1),"")</f>
-        <v>0.23688269506171555</v>
+        <v>0.23817010139269423</v>
       </c>
       <c r="C24" s="68">
         <f>IFERROR(IF('PyG 3 Años'!$C$9="","",C23/C20-1),"")</f>
-        <v>0.24256877306585434</v>
+        <v>0.24386209773723033</v>
       </c>
       <c r="D24" s="68">
         <f>IFERROR(IF('PyG 3 Años'!$D$9="","",D23/D20-1),"")</f>
-        <v>0.3102036085474267</v>
+        <v>0.3115673307720559</v>
       </c>
       <c r="E24" s="28" t="inlineStr">
         <is>
@@ -4510,7 +4510,7 @@
     <row r="26" ht="46" customHeight="1">
       <c r="A26" s="28" t="str">
         <f>IFERROR("Con el precio medio por invitado sin IVA de la fila de arriba necesitas "&amp;TEXT(ROUNDUP(B15,0),"0")&amp;" invitados por evento durante los "&amp;TEXT(B11,"0")&amp;" eventos del año para no perder dinero (equilibrio contable, con la amortización dentro), y "&amp;TEXT(ROUNDUP(B20,0),"0")&amp;" para que la caja aguante (equilibrio de caja: sin la amortización, que no se paga, y con la cuota del préstamo del año"&amp;IF(B12=0,"; este año sólo intereses, porque el préstamo está en carencia","")&amp;"). En las filas «Ingresos necesarios al año» tienes esas mismas cifras en euros.","")</f>
-        <v>Con el precio medio por invitado sin IVA de la fila de arriba necesitas 55 invitados por evento durante los 130 eventos del año para no perder dinero (equilibrio contable, con la amortización dentro), y 53 para que la caja aguante (equilibrio de caja: sin la amortización, que no se paga, y con la cuota del préstamo del año; este año sólo intereses, porque el préstamo está en carencia). En las filas «Ingresos necesarios al año» tienes esas mismas cifras en euros.</v>
+        <v>Con el precio medio por invitado sin IVA de la fila de arriba necesitas 54 invitados por evento durante los 130 eventos del año para no perder dinero (equilibrio contable, con la amortización dentro), y 53 para que la caja aguante (equilibrio de caja: sin la amortización, que no se paga, y con la cuota del préstamo del año; este año sólo intereses, porque el préstamo está en carencia). En las filas «Ingresos necesarios al año» tienes esas mismas cifras en euros.</v>
       </c>
       <c r="B26" s="28" t="n"/>
       <c r="C26" s="28" t="n"/>
@@ -4585,115 +4585,115 @@
     <row r="32">
       <c r="A32" s="70">
         <f>IFERROR($B$9*0.85,"")</f>
-        <v>17.4360619</v>
+        <v>17.40732</v>
       </c>
       <c r="B32" s="44">
         <f>IFERROR(IF($B$31-$A32&lt;=0,"",$B$6/($B$31-$A32)/$B$11),"")</f>
-        <v>52.31886751600316</v>
+        <v>52.27410348829658</v>
       </c>
       <c r="C32" s="44">
         <f>IFERROR(IF($C$31-$A32&lt;=0,"",$B$6/($C$31-$A32)/$B$11),"")</f>
-        <v>49.37662487859382</v>
+        <v>49.336752129067854</v>
       </c>
       <c r="D32" s="44">
         <f>IFERROR(IF($D$31-$A32&lt;=0,"",$B$6/($D$31-$A32)/$B$11),"")</f>
-        <v>46.7476872657617</v>
+        <v>46.711945803524266</v>
       </c>
       <c r="E32" s="44">
         <f>IFERROR(IF($E$31-$A32&lt;=0,"",$B$6/($E$31-$A32)/$B$11),"")</f>
-        <v>44.38454095067019</v>
+        <v>44.35232044835638</v>
       </c>
       <c r="F32" s="28" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="70">
         <f>IFERROR($B$9*0.925,"")</f>
-        <v>18.97453795</v>
+        <v>18.94326</v>
       </c>
       <c r="B33" s="44">
         <f>IFERROR(IF($B$31-$A33&lt;=0,"",$B$6/($B$31-$A33)/$B$11),"")</f>
-        <v>54.83222156256855</v>
+        <v>54.778721441083235</v>
       </c>
       <c r="C33" s="44">
         <f>IFERROR(IF($C$31-$A33&lt;=0,"",$B$6/($C$31-$A33)/$B$11),"")</f>
-        <v>51.60921042567387</v>
+        <v>51.56181216314981</v>
       </c>
       <c r="D33" s="44">
         <f>IFERROR(IF($D$31-$A33&lt;=0,"",$B$6/($D$31-$A33)/$B$11),"")</f>
-        <v>48.74405853093648</v>
+        <v>48.70177477967311</v>
       </c>
       <c r="E33" s="44">
         <f>IFERROR(IF($E$31-$A33&lt;=0,"",$B$6/($E$31-$A33)/$B$11),"")</f>
-        <v>46.18029962292676</v>
+        <v>46.14234510809992</v>
       </c>
       <c r="F33" s="28" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="70">
         <f>IFERROR($B$9*1.0,"")</f>
-        <v>20.513014</v>
+        <v>20.4792</v>
       </c>
       <c r="B34" s="44">
         <f>IFERROR(IF($B$31-$A34&lt;=0,"",$B$6/($B$31-$A34)/$B$11),"")</f>
-        <v>57.59924023874419</v>
+        <v>57.53542602976432</v>
       </c>
       <c r="C34" s="44">
         <f>IFERROR(IF($C$31-$A34&lt;=0,"",$B$6/($C$31-$A34)/$B$11),"")</f>
-        <v>54.05325168574366</v>
+        <v>53.99704898923861</v>
       </c>
       <c r="D34" s="44">
         <f>IFERROR(IF($D$31-$A34&lt;=0,"",$B$6/($D$31-$A34)/$B$11),"")</f>
-        <v>50.91854738390971</v>
+        <v>50.86867137404784</v>
       </c>
       <c r="E34" s="44">
         <f>IFERROR(IF($E$31-$A34&lt;=0,"",$B$6/($E$31-$A34)/$B$11),"")</f>
-        <v>48.127494848964254</v>
+        <v>48.08293440366123</v>
       </c>
       <c r="F34" s="28" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="70">
         <f>IFERROR($B$9*1.075,"")</f>
-        <v>22.051490049999998</v>
+        <v>22.01514</v>
       </c>
       <c r="B35" s="44">
         <f>IFERROR(IF($B$31-$A35&lt;=0,"",$B$6/($B$31-$A35)/$B$11),"")</f>
-        <v>60.66036676161395</v>
+        <v>60.58429230878571</v>
       </c>
       <c r="C35" s="44">
         <f>IFERROR(IF($C$31-$A35&lt;=0,"",$B$6/($C$31-$A35)/$B$11),"")</f>
-        <v>56.740283574435246</v>
+        <v>56.67371841503337</v>
       </c>
       <c r="D35" s="44">
         <f>IFERROR(IF($D$31-$A35&lt;=0,"",$B$6/($D$31-$A35)/$B$11),"")</f>
-        <v>53.29610454111691</v>
+        <v>53.23737104748151</v>
       </c>
       <c r="E35" s="44">
         <f>IFERROR(IF($E$31-$A35&lt;=0,"",$B$6/($E$31-$A35)/$B$11),"")</f>
-        <v>50.24612589439541</v>
+        <v>50.193919048675085</v>
       </c>
       <c r="F35" s="28" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="70">
         <f>IFERROR($B$9*1.15,"")</f>
-        <v>23.589966099999994</v>
+        <v>23.551079999999995</v>
       </c>
       <c r="B36" s="44">
         <f>IFERROR(IF($B$31-$A36&lt;=0,"",$B$6/($B$31-$A36)/$B$11),"")</f>
-        <v>64.06512436926357</v>
+        <v>63.974365139656875</v>
       </c>
       <c r="C36" s="44">
         <f>IFERROR(IF($C$31-$A36&lt;=0,"",$B$6/($C$31-$A36)/$B$11),"")</f>
-        <v>59.70843953257839</v>
+        <v>59.62959696889497</v>
       </c>
       <c r="D36" s="44">
         <f>IFERROR(IF($D$31-$A36&lt;=0,"",$B$6/($D$31-$A36)/$B$11),"")</f>
-        <v>55.906569103360006</v>
+        <v>55.83744150098733</v>
       </c>
       <c r="E36" s="44">
         <f>IFERROR(IF($E$31-$A36&lt;=0,"",$B$6/($E$31-$A36)/$B$11),"")</f>
-        <v>52.55987575544575</v>
+        <v>52.49877218066325</v>
       </c>
       <c r="F36" s="28" t="n"/>
     </row>
@@ -5033,15 +5033,15 @@
       </c>
       <c r="B9" s="32">
         <f>IFERROR(IF(B8="","",B8*'0. Supuestos'!$B$11*'0. Supuestos'!$B$13),"")</f>
-        <v>80504.55</v>
+        <v>77489.99999999999</v>
       </c>
       <c r="C9" s="32">
         <f>IFERROR(IF(C8="","",C8*'0. Supuestos'!$B$11*'0. Supuestos'!$B$13),"")</f>
-        <v>114457.02449999998</v>
+        <v>110171.09999999999</v>
       </c>
       <c r="D9" s="32">
         <f>IFERROR(IF(D8="","",D8*'0. Supuestos'!$B$11*'0. Supuestos'!$B$13),"")</f>
-        <v>152958.645</v>
+        <v>147230.99999999997</v>
       </c>
       <c r="E9" s="28" t="n"/>
       <c r="F9" s="28" t="n"/>
@@ -5054,15 +5054,15 @@
       </c>
       <c r="B10" s="32">
         <f>IFERROR(IF(B8="","",B8*'0. Supuestos'!$B$12*'0. Supuestos'!$B$14),"")</f>
-        <v>13062.420000000002</v>
+        <v>15876.000000000005</v>
       </c>
       <c r="C10" s="32">
         <f>IFERROR(IF(C8="","",C8*'0. Supuestos'!$B$12*'0. Supuestos'!$B$14),"")</f>
-        <v>18571.443800000005</v>
+        <v>22571.64000000001</v>
       </c>
       <c r="D10" s="32">
         <f>IFERROR(IF(D8="","",D8*'0. Supuestos'!$B$12*'0. Supuestos'!$B$14),"")</f>
-        <v>24818.598000000005</v>
+        <v>30164.400000000012</v>
       </c>
       <c r="E10" s="28" t="n"/>
       <c r="F10" s="28" t="n"/>
@@ -5159,15 +5159,15 @@
       </c>
       <c r="B15" s="32">
         <f>IFERROR(IF(B8="","",SUM(B9:B14)),"")</f>
-        <v>121916.97</v>
+        <v>121715.99999999999</v>
       </c>
       <c r="C15" s="32">
         <f>IFERROR(IF(C8="","",SUM(C9:C14)),"")</f>
-        <v>173334.96829999998</v>
+        <v>173049.24</v>
       </c>
       <c r="D15" s="32">
         <f>IFERROR(IF(D8="","",SUM(D9:D14)),"")</f>
-        <v>231642.243</v>
+        <v>231260.4</v>
       </c>
       <c r="E15" s="28" t="n"/>
       <c r="F15" s="28" t="n"/>
@@ -5180,15 +5180,15 @@
       </c>
       <c r="B16" s="32">
         <f>IFERROR(IF(B8="","",B8-B15),"")</f>
-        <v>193083.03</v>
+        <v>193284.0</v>
       </c>
       <c r="C16" s="32">
         <f>IFERROR(IF(C8="","",C8-C15),"")</f>
-        <v>274515.03170000005</v>
+        <v>274800.76</v>
       </c>
       <c r="D16" s="32">
         <f>IFERROR(IF(D8="","",D8-D15),"")</f>
-        <v>366857.757</v>
+        <v>367239.6</v>
       </c>
       <c r="E16" s="28" t="n"/>
       <c r="F16" s="28" t="n"/>
@@ -5226,15 +5226,15 @@
       </c>
       <c r="B18" s="26">
         <f>IFERROR(IF(B8="","",B16-B17),"")</f>
-        <v>-35200.51000000001</v>
+        <v>-34999.54000000001</v>
       </c>
       <c r="C18" s="26">
         <f>IFERROR(IF(C8="","",C16-C17),"")</f>
-        <v>46231.49170000004</v>
+        <v>46517.22</v>
       </c>
       <c r="D18" s="26">
         <f>IFERROR(IF(D8="","",D16-D17),"")</f>
-        <v>138574.21699999998</v>
+        <v>138956.05999999997</v>
       </c>
       <c r="E18" s="28" t="n"/>
       <c r="F18" s="28" t="n"/>
@@ -5251,11 +5251,11 @@
       </c>
       <c r="C19" s="32">
         <f>IFERROR(IF(C8="","",MAX(0,C18-'0. Supuestos'!$B$42)*'0. Supuestos'!$B$37),"")</f>
-        <v>6934.723755000006</v>
+        <v>6977.583</v>
       </c>
       <c r="D19" s="32">
         <f>IFERROR(IF(D8="","",MAX(0,D18-'0. Supuestos'!$B$42)*'0. Supuestos'!$B$37),"")</f>
-        <v>20786.132549999995</v>
+        <v>20843.408999999996</v>
       </c>
       <c r="E19" s="28" t="inlineStr">
         <is>
@@ -5272,15 +5272,15 @@
       </c>
       <c r="B20" s="26">
         <f>IFERROR(IF(B8="","",B18-B19),"")</f>
-        <v>-35200.51000000001</v>
+        <v>-34999.54000000001</v>
       </c>
       <c r="C20" s="26">
         <f>IFERROR(IF(C8="","",C18-C19),"")</f>
-        <v>39296.767945000036</v>
+        <v>39539.637</v>
       </c>
       <c r="D20" s="26">
         <f>IFERROR(IF(D8="","",D18-D19),"")</f>
-        <v>117788.08444999998</v>
+        <v>118112.65099999997</v>
       </c>
       <c r="E20" s="28" t="n"/>
       <c r="F20" s="28" t="n"/>
@@ -5293,15 +5293,15 @@
       </c>
       <c r="B21" s="44">
         <f>IFERROR(IF(B8="","",IF(B6-B15/(B5*B7)&lt;=0,"",B17/(B6-B15/(B5*B7))/B7)),"")</f>
-        <v>70.93845792662358</v>
+        <v>70.8646985782579</v>
       </c>
       <c r="C21" s="44">
         <f>IFERROR(IF(C8="","",IF(C6-C15/(C5*C7)&lt;=0,"",C17/(C6-C15/(C5*C7))/C7)),"")</f>
-        <v>54.05325168574366</v>
+        <v>53.99704898923861</v>
       </c>
       <c r="D21" s="44">
         <f>IFERROR(IF(D8="","",IF(D6-D15/(D5*D7)&lt;=0,"",D17/(D6-D15/(D5*D7))/D7)),"")</f>
-        <v>43.55870223564607</v>
+        <v>43.513411407702215</v>
       </c>
       <c r="E21" s="28" t="n"/>
       <c r="F21" s="28" t="n"/>
@@ -5376,15 +5376,15 @@
       </c>
       <c r="B25" s="26">
         <f>IFERROR(IF(B8="","",'Inversión Inicial'!$B$25+B20+'PyG 3 Años'!$B$36-'Financiación'!$B$45),"")</f>
-        <v>26627.249999999993</v>
+        <v>26828.219999999994</v>
       </c>
       <c r="C25" s="26">
         <f>IFERROR(IF(C8="","",'Inversión Inicial'!$B$25+C20+'PyG 3 Años'!$B$36-'Financiación'!$B$45),"")</f>
-        <v>101124.52794500004</v>
+        <v>101367.397</v>
       </c>
       <c r="D25" s="26">
         <f>IFERROR(IF(D8="","",'Inversión Inicial'!$B$25+D20+'PyG 3 Años'!$B$36-'Financiación'!$B$45),"")</f>
-        <v>179615.84444999998</v>
+        <v>179940.41099999996</v>
       </c>
       <c r="E25" s="25" t="inlineStr">
         <is>
@@ -5402,7 +5402,7 @@
       <c r="B26" s="28" t="n"/>
       <c r="C26" s="32">
         <f>IFERROR(IF(C8="","",'Tesorería 12 meses'!$M$22),"")</f>
-        <v>93173.37980435265</v>
+        <v>93243.88811842892</v>
       </c>
       <c r="D26" s="28" t="n"/>
       <c r="E26" s="28" t="inlineStr">
@@ -6342,7 +6342,7 @@
       </c>
       <c r="B18" s="68">
         <f>IFERROR(IF('PyG 3 Años'!$B$53="","",'PyG 3 Años'!$B$53),"")</f>
-        <v>0.29703799999999997</v>
+        <v>0.2964</v>
       </c>
       <c r="C18" s="68">
         <f>IFERROR(IF('PyG 3 Años'!$E$53="","",'PyG 3 Años'!$E$53),"")</f>
@@ -6402,7 +6402,7 @@
       </c>
       <c r="B21" s="68">
         <f>IFERROR(IF('PyG 3 Años'!$B$56="","",'PyG 3 Años'!$B$56),"")</f>
-        <v>0.08774537891034953</v>
+        <v>0.08828767891034946</v>
       </c>
       <c r="C21" s="68">
         <f>IFERROR(IF('PyG 3 Años'!$E$56="","",'PyG 3 Años'!$E$56),"")</f>
@@ -6422,7 +6422,7 @@
       </c>
       <c r="B22" s="68">
         <f>IFERROR(IF('PyG 3 Años'!$B$51="","",'PyG 3 Años'!$B$51),"")</f>
-        <v>0.6129620000000001</v>
+        <v>0.6136</v>
       </c>
       <c r="C22" s="68">
         <f>IFERROR(IF('PyG 3 Años'!$E$51="","",'PyG 3 Años'!$E$51),"")</f>
@@ -6516,7 +6516,7 @@
       </c>
       <c r="B29" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$48="","",'PyG 3 Años'!$B$48),"")</f>
-        <v>39296.767945000036</v>
+        <v>39539.637</v>
       </c>
       <c r="C29" s="28" t="n"/>
       <c r="D29" s="28" t="n"/>
@@ -6530,7 +6530,7 @@
       </c>
       <c r="B30" s="44">
         <f>IFERROR(IF('Punto Equilibrio'!$B$15="","",'Punto Equilibrio'!$B$15),"")</f>
-        <v>54.05325168574366</v>
+        <v>53.99704898923861</v>
       </c>
       <c r="C30" s="28" t="n"/>
       <c r="D30" s="28" t="n"/>
@@ -7559,55 +7559,55 @@
       </c>
       <c r="B9" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",('PyG 3 Años'!$B$9+'PyG 3 Años'!$B$9*SUMPRODUCT('PyG 3 Años'!$E$10:$E$11,'PyG 3 Años'!$G$10:$G$11))*B7*(1-MIN(30,'0. Supuestos'!$B$58)/30)),"")</f>
-        <v>1963.5983748773563</v>
+        <v>1963.8018529997642</v>
       </c>
       <c r="C9" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",('PyG 3 Años'!$B$9+'PyG 3 Años'!$B$9*SUMPRODUCT('PyG 3 Años'!$E$10:$E$11,'PyG 3 Años'!$G$10:$G$11))*(C7*(1-MIN(30,'0. Supuestos'!$B$58)/30)+B7*MIN(30,'0. Supuestos'!$B$58)/30)),"")</f>
-        <v>12959.749274190552</v>
+        <v>12961.092229798445</v>
       </c>
       <c r="D9" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",('PyG 3 Años'!$B$9+'PyG 3 Años'!$B$9*SUMPRODUCT('PyG 3 Años'!$E$10:$E$11,'PyG 3 Años'!$G$10:$G$11))*(D7*(1-MIN(30,'0. Supuestos'!$B$58)/30)+C7*MIN(30,'0. Supuestos'!$B$58)/30)),"")</f>
-        <v>20269.690497029438</v>
+        <v>20271.790946193025</v>
       </c>
       <c r="E9" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",('PyG 3 Años'!$B$9+'PyG 3 Años'!$B$9*SUMPRODUCT('PyG 3 Años'!$E$10:$E$11,'PyG 3 Años'!$G$10:$G$11))*(E7*(1-MIN(30,'0. Supuestos'!$B$58)/30)+D7*MIN(30,'0. Supuestos'!$B$58)/30)),"")</f>
-        <v>28293.667492551</v>
+        <v>28296.59942731479</v>
       </c>
       <c r="F9" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",('PyG 3 Años'!$B$9+'PyG 3 Años'!$B$9*SUMPRODUCT('PyG 3 Años'!$E$10:$E$11,'PyG 3 Años'!$G$10:$G$11))*(F7*(1-MIN(30,'0. Supuestos'!$B$58)/30)+E7*MIN(30,'0. Supuestos'!$B$58)/30)),"")</f>
-        <v>35974.014772469025</v>
+        <v>35977.7425841616</v>
       </c>
       <c r="G9" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",('PyG 3 Años'!$B$9+'PyG 3 Años'!$B$9*SUMPRODUCT('PyG 3 Años'!$E$10:$E$11,'PyG 3 Años'!$G$10:$G$11))*(G7*(1-MIN(30,'0. Supuestos'!$B$58)/30)+F7*MIN(30,'0. Supuestos'!$B$58)/30)),"")</f>
-        <v>53351.860390133625</v>
+        <v>53357.388983209516</v>
       </c>
       <c r="H9" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",('PyG 3 Años'!$B$9+'PyG 3 Años'!$B$9*SUMPRODUCT('PyG 3 Años'!$E$10:$E$11,'PyG 3 Años'!$G$10:$G$11))*(H7*(1-MIN(30,'0. Supuestos'!$B$58)/30)+G7*MIN(30,'0. Supuestos'!$B$58)/30)),"")</f>
-        <v>61585.58539388072</v>
+        <v>61591.967207719885</v>
       </c>
       <c r="I9" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",('PyG 3 Años'!$B$9+'PyG 3 Años'!$B$9*SUMPRODUCT('PyG 3 Años'!$E$10:$E$11,'PyG 3 Años'!$G$10:$G$11))*(I7*(1-MIN(30,'0. Supuestos'!$B$58)/30)+H7*MIN(30,'0. Supuestos'!$B$58)/30)),"")</f>
-        <v>44627.2357926672</v>
+        <v>44631.8602954492</v>
       </c>
       <c r="J9" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",('PyG 3 Años'!$B$9+'PyG 3 Años'!$B$9*SUMPRODUCT('PyG 3 Años'!$E$10:$E$11,'PyG 3 Años'!$G$10:$G$11))*(J7*(1-MIN(30,'0. Supuestos'!$B$58)/30)+I7*MIN(30,'0. Supuestos'!$B$58)/30)),"")</f>
-        <v>32131.609770720377</v>
+        <v>32134.93941272342</v>
       </c>
       <c r="K9" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",('PyG 3 Años'!$B$9+'PyG 3 Años'!$B$9*SUMPRODUCT('PyG 3 Años'!$E$10:$E$11,'PyG 3 Años'!$G$10:$G$11))*(K7*(1-MIN(30,'0. Supuestos'!$B$58)/30)+J7*MIN(30,'0. Supuestos'!$B$58)/30)),"")</f>
-        <v>58015.40653046735</v>
+        <v>58021.418384083954</v>
       </c>
       <c r="L9" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",('PyG 3 Años'!$B$9+'PyG 3 Años'!$B$9*SUMPRODUCT('PyG 3 Años'!$E$10:$E$11,'PyG 3 Años'!$G$10:$G$11))*(L7*(1-MIN(30,'0. Supuestos'!$B$58)/30)+K7*MIN(30,'0. Supuestos'!$B$58)/30)),"")</f>
-        <v>50875.048803640595</v>
+        <v>50880.32073681208</v>
       </c>
       <c r="M9" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",('PyG 3 Años'!$B$9+'PyG 3 Años'!$B$9*SUMPRODUCT('PyG 3 Años'!$E$10:$E$11,'PyG 3 Años'!$G$10:$G$11))*(M7*(1-MIN(30,'0. Supuestos'!$B$58)/30)+L7*MIN(30,'0. Supuestos'!$B$58)/30)),"")</f>
-        <v>41503.32928718049</v>
+        <v>41507.63007476775</v>
       </c>
       <c r="N9" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",SUM(B9:M9)),"")</f>
-        <v>441550.7963798077</v>
+        <v>441596.5521352335</v>
       </c>
       <c r="O9" s="28" t="inlineStr">
         <is>
@@ -7648,51 +7648,51 @@
       </c>
       <c r="C11" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",-('PyG 3 Años'!$B$13*(1+'PyG 3 Años'!$G$13)+'PyG 3 Años'!$B$14*(1+'PyG 3 Años'!$G$14)+'PyG 3 Años'!$B$15*(1+'PyG 3 Años'!$G$15)+'PyG 3 Años'!$B$16*(1+'PyG 3 Años'!$G$16)+'PyG 3 Años'!$B$17*(1+'PyG 3 Años'!$G$17)+'PyG 3 Años'!$B$18*(1+'PyG 3 Años'!$G$18))*(C7*(1-MIN(30,'0. Supuestos'!$B$59)/30)+B7*MIN(30,'0. Supuestos'!$B$59)/30)),"")</f>
-        <v>-4684.213080846852</v>
+        <v>-4683.536907393926</v>
       </c>
       <c r="D11" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",-('PyG 3 Años'!$B$13*(1+'PyG 3 Años'!$G$13)+'PyG 3 Años'!$B$14*(1+'PyG 3 Años'!$G$14)+'PyG 3 Años'!$B$15*(1+'PyG 3 Años'!$G$15)+'PyG 3 Años'!$B$16*(1+'PyG 3 Años'!$G$16)+'PyG 3 Años'!$B$17*(1+'PyG 3 Años'!$G$17)+'PyG 3 Años'!$B$18*(1+'PyG 3 Años'!$G$18))*(D7*(1-MIN(30,'0. Supuestos'!$B$59)/30)+C7*MIN(30,'0. Supuestos'!$B$59)/30)),"")</f>
-        <v>-7494.740929354963</v>
+        <v>-7493.659051830283</v>
       </c>
       <c r="E11" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",-('PyG 3 Años'!$B$13*(1+'PyG 3 Años'!$G$13)+'PyG 3 Años'!$B$14*(1+'PyG 3 Años'!$G$14)+'PyG 3 Años'!$B$15*(1+'PyG 3 Años'!$G$15)+'PyG 3 Años'!$B$16*(1+'PyG 3 Años'!$G$16)+'PyG 3 Años'!$B$17*(1+'PyG 3 Años'!$G$17)+'PyG 3 Años'!$B$18*(1+'PyG 3 Años'!$G$18))*(E7*(1-MIN(30,'0. Supuestos'!$B$59)/30)+D7*MIN(30,'0. Supuestos'!$B$59)/30)),"")</f>
-        <v>-10880.149474148822</v>
+        <v>-10878.57890762862</v>
       </c>
       <c r="F11" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",-('PyG 3 Años'!$B$13*(1+'PyG 3 Años'!$G$13)+'PyG 3 Años'!$B$14*(1+'PyG 3 Años'!$G$14)+'PyG 3 Años'!$B$15*(1+'PyG 3 Años'!$G$15)+'PyG 3 Años'!$B$16*(1+'PyG 3 Años'!$G$16)+'PyG 3 Años'!$B$17*(1+'PyG 3 Años'!$G$17)+'PyG 3 Años'!$B$18*(1+'PyG 3 Años'!$G$18))*(F7*(1-MIN(30,'0. Supuestos'!$B$59)/30)+E7*MIN(30,'0. Supuestos'!$B$59)/30)),"")</f>
-        <v>-13094.50474873097</v>
+        <v>-13092.614536578476</v>
       </c>
       <c r="G11" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",-('PyG 3 Años'!$B$13*(1+'PyG 3 Años'!$G$13)+'PyG 3 Años'!$B$14*(1+'PyG 3 Años'!$G$14)+'PyG 3 Años'!$B$15*(1+'PyG 3 Años'!$G$15)+'PyG 3 Años'!$B$16*(1+'PyG 3 Años'!$G$16)+'PyG 3 Años'!$B$17*(1+'PyG 3 Años'!$G$17)+'PyG 3 Años'!$B$18*(1+'PyG 3 Años'!$G$18))*(G7*(1-MIN(30,'0. Supuestos'!$B$59)/30)+F7*MIN(30,'0. Supuestos'!$B$59)/30)),"")</f>
-        <v>-20344.389085223484</v>
+        <v>-20341.4523409768</v>
       </c>
       <c r="H11" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",-('PyG 3 Años'!$B$13*(1+'PyG 3 Años'!$G$13)+'PyG 3 Años'!$B$14*(1+'PyG 3 Años'!$G$14)+'PyG 3 Años'!$B$15*(1+'PyG 3 Años'!$G$15)+'PyG 3 Años'!$B$16*(1+'PyG 3 Años'!$G$16)+'PyG 3 Años'!$B$17*(1+'PyG 3 Años'!$G$17)+'PyG 3 Años'!$B$18*(1+'PyG 3 Años'!$G$18))*(H7*(1-MIN(30,'0. Supuestos'!$B$59)/30)+G7*MIN(30,'0. Supuestos'!$B$59)/30)),"")</f>
-        <v>-25550.25316825555</v>
+        <v>-25546.564949421416</v>
       </c>
       <c r="I11" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",-('PyG 3 Años'!$B$13*(1+'PyG 3 Años'!$G$13)+'PyG 3 Años'!$B$14*(1+'PyG 3 Años'!$G$14)+'PyG 3 Años'!$B$15*(1+'PyG 3 Años'!$G$15)+'PyG 3 Años'!$B$16*(1+'PyG 3 Años'!$G$16)+'PyG 3 Años'!$B$17*(1+'PyG 3 Años'!$G$17)+'PyG 3 Años'!$B$18*(1+'PyG 3 Años'!$G$18))*(I7*(1-MIN(30,'0. Supuestos'!$B$59)/30)+H7*MIN(30,'0. Supuestos'!$B$59)/30)),"")</f>
-        <v>-19162.689876191664</v>
+        <v>-19159.923712066062</v>
       </c>
       <c r="J11" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",-('PyG 3 Años'!$B$13*(1+'PyG 3 Años'!$G$13)+'PyG 3 Años'!$B$14*(1+'PyG 3 Años'!$G$14)+'PyG 3 Años'!$B$15*(1+'PyG 3 Años'!$G$15)+'PyG 3 Años'!$B$16*(1+'PyG 3 Años'!$G$16)+'PyG 3 Años'!$B$17*(1+'PyG 3 Años'!$G$17)+'PyG 3 Años'!$B$18*(1+'PyG 3 Años'!$G$18))*(J7*(1-MIN(30,'0. Supuestos'!$B$59)/30)+I7*MIN(30,'0. Supuestos'!$B$59)/30)),"")</f>
-        <v>-10645.93882010648</v>
+        <v>-10644.402062258923</v>
       </c>
       <c r="K11" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",-('PyG 3 Años'!$B$13*(1+'PyG 3 Años'!$G$13)+'PyG 3 Años'!$B$14*(1+'PyG 3 Años'!$G$14)+'PyG 3 Años'!$B$15*(1+'PyG 3 Años'!$G$15)+'PyG 3 Años'!$B$16*(1+'PyG 3 Años'!$G$16)+'PyG 3 Años'!$B$17*(1+'PyG 3 Años'!$G$17)+'PyG 3 Años'!$B$18*(1+'PyG 3 Años'!$G$18))*(K7*(1-MIN(30,'0. Supuestos'!$B$59)/30)+J7*MIN(30,'0. Supuestos'!$B$59)/30)),"")</f>
-        <v>-23421.065404234254</v>
+        <v>-23417.68453696963</v>
       </c>
       <c r="L11" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",-('PyG 3 Años'!$B$13*(1+'PyG 3 Años'!$G$13)+'PyG 3 Años'!$B$14*(1+'PyG 3 Años'!$G$14)+'PyG 3 Años'!$B$15*(1+'PyG 3 Años'!$G$15)+'PyG 3 Años'!$B$16*(1+'PyG 3 Años'!$G$16)+'PyG 3 Años'!$B$17*(1+'PyG 3 Años'!$G$17)+'PyG 3 Años'!$B$18*(1+'PyG 3 Años'!$G$18))*(L7*(1-MIN(30,'0. Supuestos'!$B$59)/30)+K7*MIN(30,'0. Supuestos'!$B$59)/30)),"")</f>
-        <v>-21291.87764021296</v>
+        <v>-21288.804124517847</v>
       </c>
       <c r="M11" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",-('PyG 3 Años'!$B$13*(1+'PyG 3 Años'!$G$13)+'PyG 3 Años'!$B$14*(1+'PyG 3 Años'!$G$14)+'PyG 3 Años'!$B$15*(1+'PyG 3 Años'!$G$15)+'PyG 3 Años'!$B$16*(1+'PyG 3 Años'!$G$16)+'PyG 3 Años'!$B$17*(1+'PyG 3 Años'!$G$17)+'PyG 3 Años'!$B$18*(1+'PyG 3 Años'!$G$18))*(M7*(1-MIN(30,'0. Supuestos'!$B$59)/30)+L7*MIN(30,'0. Supuestos'!$B$59)/30)),"")</f>
-        <v>-14904.314348149072</v>
+        <v>-14902.162887162493</v>
       </c>
       <c r="N11" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",SUM(B11:M11)),"")</f>
-        <v>-171474.13657545505</v>
+        <v>-171449.38401680448</v>
       </c>
       <c r="O11" s="28" t="str">
         <f>IFERROR("Materia prima, consumibles, comisiones e imprevistos, cada uno con SU tipo de IVA (la columna del P&amp;L) y con los días de pago a proveedor de Supuestos."&amp;IF('0. Supuestos'!$B$59=0,""," Con "&amp;TEXT('0. Supuestos'!$B$59,"0")&amp;" días de pago, las primeras compras se pagan ya en el año siguiente: la columna «Año» de esta fila recoge "&amp;TEXT(MAX(0,12-ROUNDUP('0. Supuestos'!$B$59/30,0)),"0")&amp;" mensualidades de compra, no el coste del ejercicio."),"")</f>
@@ -7955,59 +7955,59 @@
       </c>
       <c r="B16" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",'PyG 3 Años'!$B$9*B7*SUMPRODUCT('PyG 3 Años'!$E$10:$E$11,'PyG 3 Años'!$G$10:$G$11)),"")</f>
-        <v>1076.2064278918347</v>
+        <v>1077.4272966262836</v>
       </c>
       <c r="C16" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",'PyG 3 Años'!$B$9*C7*SUMPRODUCT('PyG 3 Años'!$E$10:$E$11,'PyG 3 Años'!$G$10:$G$11)),"")</f>
-        <v>1721.9302846269354</v>
+        <v>1723.8836746020538</v>
       </c>
       <c r="D16" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",'PyG 3 Años'!$B$9*D7*SUMPRODUCT('PyG 3 Años'!$E$10:$E$11,'PyG 3 Años'!$G$10:$G$11)),"")</f>
-        <v>2499.7340211487617</v>
+        <v>2502.5697662546863</v>
       </c>
       <c r="E16" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",'PyG 3 Años'!$B$9*E7*SUMPRODUCT('PyG 3 Años'!$E$10:$E$11,'PyG 3 Años'!$G$10:$G$11)),"")</f>
-        <v>3008.486150697629</v>
+        <v>3011.8990337507475</v>
       </c>
       <c r="F16" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",'PyG 3 Años'!$B$9*F7*SUMPRODUCT('PyG 3 Años'!$E$10:$E$11,'PyG 3 Años'!$G$10:$G$11)),"")</f>
-        <v>4674.160190230218</v>
+        <v>4679.462645120064</v>
       </c>
       <c r="G16" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",'PyG 3 Años'!$B$9*G7*SUMPRODUCT('PyG 3 Años'!$E$10:$E$11,'PyG 3 Años'!$G$10:$G$11)),"")</f>
-        <v>5870.216879410007</v>
+        <v>5876.876163416092</v>
       </c>
       <c r="H16" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",'PyG 3 Años'!$B$9*H7*SUMPRODUCT('PyG 3 Años'!$E$10:$E$11,'PyG 3 Años'!$G$10:$G$11)),"")</f>
-        <v>4402.662659557505</v>
+        <v>4407.657122562069</v>
       </c>
       <c r="I16" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",'PyG 3 Años'!$B$9*I7*SUMPRODUCT('PyG 3 Años'!$E$10:$E$11,'PyG 3 Años'!$G$10:$G$11)),"")</f>
-        <v>2445.92369975417</v>
+        <v>2448.6984014233717</v>
       </c>
       <c r="J16" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",'PyG 3 Años'!$B$9*J7*SUMPRODUCT('PyG 3 Años'!$E$10:$E$11,'PyG 3 Años'!$G$10:$G$11)),"")</f>
-        <v>5381.032139459174</v>
+        <v>5387.136483131419</v>
       </c>
       <c r="K16" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",'PyG 3 Años'!$B$9*K7*SUMPRODUCT('PyG 3 Años'!$E$10:$E$11,'PyG 3 Años'!$G$10:$G$11)),"")</f>
-        <v>4891.84739950834</v>
+        <v>4897.396802846743</v>
       </c>
       <c r="L16" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",'PyG 3 Años'!$B$9*L7*SUMPRODUCT('PyG 3 Años'!$E$10:$E$11,'PyG 3 Años'!$G$10:$G$11)),"")</f>
-        <v>3424.2931796558373</v>
+        <v>3428.17776199272</v>
       </c>
       <c r="M16" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",'PyG 3 Años'!$B$9*M7*SUMPRODUCT('PyG 3 Años'!$E$10:$E$11,'PyG 3 Años'!$G$10:$G$11)),"")</f>
-        <v>5625.62450943459</v>
+        <v>5632.006323273756</v>
       </c>
       <c r="N16" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",SUM(B16:M16)),"")</f>
-        <v>45022.117541375</v>
+        <v>45073.191475</v>
       </c>
       <c r="O16" s="28" t="inlineStr">
         <is>
-          <t>Cada línea de venta a SU tipo, leído de la columna de IVA del P&amp;L: en el servicio de catering, alcohol incluido, el reducido (art. 91.Uno.2.2.º de la Ley 37/1992 del IVA); el alcohol que sale por drop-off, al general; el pan común y las harinas panificables, al superreducido (art. 91.Dos.1.1.º)</t>
+          <t>Cada línea de venta a SU tipo, leído de la columna de IVA del P&amp;L: en el servicio de catering, alcohol incluido, el reducido (art. 91.Uno.2.2.º de la Ley 37/1992 del IVA); el alcohol que sale por drop-off, al general; los servicios facturados aparte (mobiliario, carpas, decoración), al general (art. 90)</t>
         </is>
       </c>
     </row>
@@ -8019,55 +8019,55 @@
       </c>
       <c r="B17" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",'PyG 3 Años'!$B$39*B7+'PyG 3 Años'!$B$40/12),"")</f>
-        <v>1411.447737390558</v>
+        <v>1417.6015988156682</v>
       </c>
       <c r="C17" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",'PyG 3 Años'!$B$39*C7+'PyG 3 Años'!$B$40/12),"")</f>
-        <v>1735.9413798248927</v>
+        <v>1745.787558105069</v>
       </c>
       <c r="D17" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",'PyG 3 Años'!$B$39*D7+'PyG 3 Años'!$B$40/12),"")</f>
-        <v>2126.8087218480687</v>
+        <v>2141.1024636127563</v>
       </c>
       <c r="E17" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",'PyG 3 Años'!$B$39*E7+'PyG 3 Años'!$B$40/12),"")</f>
-        <v>2382.470379523605</v>
+        <v>2399.6732194165265</v>
       </c>
       <c r="F17" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",'PyG 3 Años'!$B$39*F7+'PyG 3 Años'!$B$40/12),"")</f>
-        <v>3219.5164798939913</v>
+        <v>3246.24381894714</v>
       </c>
       <c r="G17" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",'PyG 3 Años'!$B$39*G7+'PyG 3 Años'!$B$40/12),"")</f>
-        <v>3820.5672039484975</v>
+        <v>3854.1337208127347</v>
       </c>
       <c r="H17" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",'PyG 3 Años'!$B$39*H7+'PyG 3 Años'!$B$40/12),"")</f>
-        <v>3083.0816529613735</v>
+        <v>3108.256540609551</v>
       </c>
       <c r="I17" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",'PyG 3 Años'!$B$39*I7+'PyG 3 Años'!$B$40/12),"")</f>
-        <v>2099.767584978541</v>
+        <v>2113.7536336719727</v>
       </c>
       <c r="J17" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",'PyG 3 Años'!$B$39*J7+'PyG 3 Años'!$B$40/12),"")</f>
-        <v>3574.73868695279</v>
+        <v>3605.5079940783403</v>
       </c>
       <c r="K17" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",'PyG 3 Años'!$B$39*K7+'PyG 3 Años'!$B$40/12),"")</f>
-        <v>3328.9101699570815</v>
+        <v>3356.8822673439454</v>
       </c>
       <c r="L17" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",'PyG 3 Años'!$B$39*L7+'PyG 3 Años'!$B$40/12),"")</f>
-        <v>2591.424618969957</v>
+        <v>2611.005087140762</v>
       </c>
       <c r="M17" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",'PyG 3 Años'!$B$39*M7+'PyG 3 Años'!$B$40/12),"")</f>
-        <v>3697.652945450644</v>
+        <v>3729.8208574455375</v>
       </c>
       <c r="N17" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",SUM(B17:M17)),"")</f>
-        <v>33072.3275617</v>
+        <v>33329.76876</v>
       </c>
       <c r="O17" s="28" t="inlineStr">
         <is>
@@ -8092,13 +8092,13 @@
       <c r="G18" s="28" t="n"/>
       <c r="H18" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",MAX(0,-E19)),"")</f>
-        <v>14651.127105395986</v>
+        <v>14675.41088305047</v>
       </c>
       <c r="I18" s="28" t="n"/>
       <c r="J18" s="28" t="n"/>
       <c r="K18" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",MAX(0,-H19)),"")</f>
-        <v>10520.817948424226</v>
+        <v>10607.223799939968</v>
       </c>
       <c r="L18" s="28" t="n"/>
       <c r="M18" s="28" t="n"/>
@@ -8120,19 +8120,19 @@
       <c r="D19" s="28" t="n"/>
       <c r="E19" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",SUM(B16:D16)-SUM(B17:D17)-E18),"")</f>
-        <v>-14651.127105395986</v>
+        <v>-14675.41088305047</v>
       </c>
       <c r="F19" s="28" t="n"/>
       <c r="G19" s="28" t="n"/>
       <c r="H19" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",SUM(E16:G16)-SUM(E17:G17)-H18),"")</f>
-        <v>-10520.817948424226</v>
+        <v>-10607.223799939968</v>
       </c>
       <c r="I19" s="28" t="n"/>
       <c r="J19" s="28" t="n"/>
       <c r="K19" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",SUM(H16:J16)-SUM(H17:J17)-K18),"")</f>
-        <v>-7048.787374546082</v>
+        <v>-7191.249961182972</v>
       </c>
       <c r="L19" s="28" t="n"/>
       <c r="M19" s="28" t="n"/>
@@ -8188,55 +8188,55 @@
       </c>
       <c r="B21" s="26">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",SUM(B9:B15)+IF(B20="",0,B20)),"")</f>
-        <v>-15464.30329178931</v>
+        <v>-15464.099813666904</v>
       </c>
       <c r="C21" s="26">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",SUM(C9:C15)+IF(C20="",0,C20)),"")</f>
-        <v>-9152.365473322967</v>
+        <v>-9150.34634426215</v>
       </c>
       <c r="D21" s="26">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",SUM(D9:D15)+IF(D20="",0,D20)),"")</f>
-        <v>-4652.952098992192</v>
+        <v>-4649.769772303926</v>
       </c>
       <c r="E21" s="26">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",SUM(E9:E15)+IF(E20="",0,E20)),"")</f>
-        <v>-14.38364826448742</v>
+        <v>-9.881146980496851</v>
       </c>
       <c r="F21" s="26">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",SUM(F9:F15)+IF(F20="",0,F20)),"")</f>
-        <v>5451.608357071385</v>
+        <v>5457.226380916454</v>
       </c>
       <c r="G21" s="26">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",SUM(G9:G15)+IF(G20="",0,G20)),"")</f>
-        <v>15579.569638243473</v>
+        <v>15588.034975566046</v>
       </c>
       <c r="H21" s="26">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",SUM(H9:H15)+IF(H20="",0,H20)),"")</f>
-        <v>6980.570558958501</v>
+        <v>6990.6405916318</v>
       </c>
       <c r="I21" s="26">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",SUM(I9:I15)+IF(I20="",0,I20)),"")</f>
-        <v>8036.644249808865</v>
+        <v>8044.034916716471</v>
       </c>
       <c r="J21" s="26">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",SUM(J9:J15)+IF(J20="",0,J20)),"")</f>
-        <v>4057.7692839472293</v>
+        <v>4062.6356837978274</v>
       </c>
       <c r="K21" s="26">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",SUM(K9:K15)+IF(K20="",0,K20)),"")</f>
-        <v>17166.439459566423</v>
+        <v>17175.832180447655</v>
       </c>
       <c r="L21" s="26">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",SUM(L9:L15)+IF(L20="",0,L20)),"")</f>
-        <v>12155.269496760968</v>
+        <v>12163.614945627563</v>
       </c>
       <c r="M21" s="26">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",SUM(M9:M15)+IF(M20="",0,M20)),"")</f>
-        <v>-2455.746727635251</v>
+        <v>-2449.294479061409</v>
       </c>
       <c r="N21" s="26">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",SUM(B21:M21)),"")</f>
-        <v>37688.11980435264</v>
+        <v>37758.628118428926</v>
       </c>
       <c r="O21" s="28" t="n"/>
     </row>
@@ -8248,51 +8248,51 @@
       </c>
       <c r="B22" s="26">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",'Inversión Inicial'!$B$25+B21),"")</f>
-        <v>40020.956708210695</v>
+        <v>40021.1601863331</v>
       </c>
       <c r="C22" s="26">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",B22+C21),"")</f>
-        <v>30868.59123488773</v>
+        <v>30870.81384207095</v>
       </c>
       <c r="D22" s="26">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",C22+D21),"")</f>
-        <v>26215.639135895537</v>
+        <v>26221.044069767024</v>
       </c>
       <c r="E22" s="26">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",D22+E21),"")</f>
-        <v>26201.25548763105</v>
+        <v>26211.162922786527</v>
       </c>
       <c r="F22" s="26">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",E22+F21),"")</f>
-        <v>31652.863844702435</v>
+        <v>31668.38930370298</v>
       </c>
       <c r="G22" s="26">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",F22+G21),"")</f>
-        <v>47232.43348294591</v>
+        <v>47256.42427926903</v>
       </c>
       <c r="H22" s="26">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",G22+H21),"")</f>
-        <v>54213.00404190441</v>
+        <v>54247.064870900824</v>
       </c>
       <c r="I22" s="26">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",H22+I21),"")</f>
-        <v>62249.648291713274</v>
+        <v>62291.09978761729</v>
       </c>
       <c r="J22" s="26">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",I22+J21),"")</f>
-        <v>66307.41757566051</v>
+        <v>66353.73547141512</v>
       </c>
       <c r="K22" s="26">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",J22+K21),"")</f>
-        <v>83473.85703522693</v>
+        <v>83529.56765186277</v>
       </c>
       <c r="L22" s="26">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",K22+L21),"")</f>
-        <v>95629.1265319879</v>
+        <v>95693.18259749033</v>
       </c>
       <c r="M22" s="26">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",L22+M21),"")</f>
-        <v>93173.37980435265</v>
+        <v>93243.88811842892</v>
       </c>
       <c r="N22" s="28" t="n"/>
       <c r="O22" s="28" t="n"/>
@@ -8305,7 +8305,7 @@
       </c>
       <c r="B23" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",IF(COUNT(B22:M22)=0,"",MIN(B22:M22))),"")</f>
-        <v>26201.25548763105</v>
+        <v>26211.162922786527</v>
       </c>
       <c r="C23" s="28" t="n"/>
       <c r="D23" s="28" t="inlineStr">
@@ -8382,7 +8382,7 @@
       </c>
       <c r="B26" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",'PyG 3 Años'!$B$48+'PyG 3 Años'!$B$36+'Financiación'!$B$44),"")</f>
-        <v>52854.267945000036</v>
+        <v>53097.137</v>
       </c>
       <c r="C26" s="28" t="n"/>
       <c r="D26" s="28" t="inlineStr">
@@ -8410,7 +8410,7 @@
       </c>
       <c r="B27" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",'PyG 3 Años'!$C$48+'PyG 3 Años'!$C$36+'Financiación'!$B$46),"")</f>
-        <v>75754.80117840006</v>
+        <v>76026.81452000001</v>
       </c>
       <c r="C27" s="28" t="n"/>
       <c r="D27" s="28" t="inlineStr">
@@ -8438,7 +8438,7 @@
       </c>
       <c r="B28" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",'PyG 3 Años'!$D$48+'PyG 3 Años'!$D$36+'Financiación'!$B$48),"")</f>
-        <v>82068.08096104859</v>
+        <v>82327.29367480858</v>
       </c>
       <c r="C28" s="28" t="n"/>
       <c r="D28" s="28" t="inlineStr">
@@ -8466,7 +8466,7 @@
       </c>
       <c r="B29" s="32">
         <f>IFERROR(IF('PyG 3 Años'!$B$9="","",N21+'Financiación'!$B$44+'Financiación'!$B$45),"")</f>
-        <v>44903.11980435264</v>
+        <v>44973.628118428926</v>
       </c>
       <c r="C29" s="28" t="n"/>
       <c r="D29" s="28" t="inlineStr">
@@ -9825,11 +9825,11 @@
       </c>
       <c r="G27" s="70">
         <f>IFERROR(IF(E27="","",'PyG 3 Años'!$B$41-'PyG 3 Años'!$B$46+'PyG 3 Años'!$B$36+'PyG 3 Años'!$B$37),"")</f>
-        <v>52854.267945000036</v>
+        <v>53097.137</v>
       </c>
       <c r="H27" s="61">
         <f>IFERROR(IF(OR(E27="",E27=0),"",G27/E27),"")</f>
-        <v>7.3256088627858675</v>
+        <v>7.3592705474705475</v>
       </c>
     </row>
     <row r="28">
@@ -9858,11 +9858,11 @@
       </c>
       <c r="G28" s="70">
         <f>IFERROR(IF(E28="","",'PyG 3 Años'!$C$41-'PyG 3 Años'!$C$46+'PyG 3 Años'!$C$36+'PyG 3 Años'!$C$37),"")</f>
-        <v>75754.80117840006</v>
+        <v>76026.81452000001</v>
       </c>
       <c r="H28" s="61">
         <f>IFERROR(IF(OR(E28="",E28=0),"",G28/E28),"")</f>
-        <v>2.8361501765531267</v>
+        <v>2.8463339625944464</v>
       </c>
     </row>
     <row r="29">
@@ -9891,11 +9891,11 @@
       </c>
       <c r="G29" s="70">
         <f>IFERROR(IF(E29="","",'PyG 3 Años'!$D$41-'PyG 3 Años'!$D$46+'PyG 3 Años'!$D$36+'PyG 3 Años'!$D$37),"")</f>
-        <v>82068.08096104859</v>
+        <v>82327.29367480858</v>
       </c>
       <c r="H29" s="61">
         <f>IFERROR(IF(OR(E29="",E29=0),"",G29/E29),"")</f>
-        <v>3.072510239435759</v>
+        <v>3.0822147884869</v>
       </c>
     </row>
     <row r="30">
@@ -9924,11 +9924,11 @@
       </c>
       <c r="G30" s="70">
         <f>IFERROR(IF(E30="","",'PyG 3 Años'!$D$41-'PyG 3 Años'!$D$46+'PyG 3 Años'!$D$36+'PyG 3 Años'!$D$37),"")</f>
-        <v>82068.08096104859</v>
+        <v>82327.29367480858</v>
       </c>
       <c r="H30" s="61">
         <f>IFERROR(IF(OR(E30="",E30=0),"",G30/E30),"")</f>
-        <v>3.072510239435759</v>
+        <v>3.0822147884869</v>
       </c>
     </row>
     <row r="31">
@@ -9957,11 +9957,11 @@
       </c>
       <c r="G31" s="70">
         <f>IFERROR(IF(E31="","",'PyG 3 Años'!$D$41-'PyG 3 Años'!$D$46+'PyG 3 Años'!$D$36+'PyG 3 Años'!$D$37),"")</f>
-        <v>82068.08096104859</v>
+        <v>82327.29367480858</v>
       </c>
       <c r="H31" s="61">
         <f>IFERROR(IF(OR(E31="",E31=0),"",G31/E31),"")</f>
-        <v>3.072510239435759</v>
+        <v>3.0822147884869</v>
       </c>
     </row>
     <row r="32">
@@ -9990,11 +9990,11 @@
       </c>
       <c r="G32" s="70">
         <f>IFERROR(IF(E32="","",'PyG 3 Años'!$D$41-'PyG 3 Años'!$D$46+'PyG 3 Años'!$D$36+'PyG 3 Años'!$D$37),"")</f>
-        <v>82068.08096104859</v>
+        <v>82327.29367480858</v>
       </c>
       <c r="H32" s="61">
         <f>IFERROR(IF(OR(E32="",E32=0),"",G32/E32),"")</f>
-        <v>3.072510239435768</v>
+        <v>3.0822147884869087</v>
       </c>
     </row>
     <row r="33">
@@ -10459,7 +10459,7 @@
       </c>
       <c r="B51" s="61">
         <f>IFERROR(('PyG 3 Años'!$B$41-'PyG 3 Años'!$B$46+'PyG 3 Años'!$B$36+B44)/(B44+B45),"")</f>
-        <v>7.3256088627858675</v>
+        <v>7.3592705474705475</v>
       </c>
       <c r="C51" s="28" t="inlineStr">
         <is>
@@ -10480,7 +10480,7 @@
       </c>
       <c r="B52" s="61">
         <f>IFERROR(('PyG 3 Años'!$C$41-'PyG 3 Años'!$C$46+'PyG 3 Años'!$C$36+B46)/(B46+B47),"")</f>
-        <v>2.8361501765531267</v>
+        <v>2.8463339625944464</v>
       </c>
       <c r="C52" s="28" t="n"/>
       <c r="D52" s="28" t="n"/>
@@ -10497,7 +10497,7 @@
       </c>
       <c r="B53" s="61">
         <f>IFERROR(('PyG 3 Años'!$D$41-'PyG 3 Años'!$D$46+'PyG 3 Años'!$D$36+B48)/(B48+B49),"")</f>
-        <v>3.072510239435759</v>
+        <v>3.0822147884869</v>
       </c>
       <c r="C53" s="28" t="n"/>
       <c r="D53" s="28" t="n"/>
@@ -10514,7 +10514,7 @@
       </c>
       <c r="B54" s="62">
         <f>IFERROR(IF(COUNT(H27:H41)=0,"",MIN(H27:H41)),"")</f>
-        <v>2.8361501765531267</v>
+        <v>2.8463339625944464</v>
       </c>
       <c r="C54" s="25" t="inlineStr">
         <is>

</xml_diff>